<commit_message>
combined pfas_table generation into one script
</commit_message>
<xml_diff>
--- a/lookup/edd_compounds.xlsx
+++ b/lookup/edd_compounds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="485" documentId="8_{8C560773-DE13-438E-BEBB-3ECB04085AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80B49985-F3E1-4B0F-B5BA-636E4BAAA87F}"/>
+  <xr:revisionPtr revIDLastSave="487" documentId="8_{8C560773-DE13-438E-BEBB-3ECB04085AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{465E1A0E-7135-45DA-B7DF-99F4AB5B2D75}"/>
   <bookViews>
-    <workbookView xWindow="-25110" yWindow="2100" windowWidth="24825" windowHeight="13935" xr2:uid="{DA70FC4B-612E-43F0-A14B-187685F0EDFF}"/>
+    <workbookView xWindow="1380" yWindow="765" windowWidth="26760" windowHeight="13875" xr2:uid="{DA70FC4B-612E-43F0-A14B-187685F0EDFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>